<commit_message>
Update latest placement portal files
</commit_message>
<xml_diff>
--- a/static/uploads/2025-2026/master_sheet.xlsx
+++ b/static/uploads/2025-2026/master_sheet.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/690d49f7c0aa36f5/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pallavai\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{316B5196-EA75-4D10-A879-C2C5EF29FF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01375714-9937-43C7-B350-564CAB968B1D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58FCC6A-F8C2-4626-B87C-94DCAD2BD36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9CB53044-4ACA-476F-BD6F-9B67AAF67AA6}"/>
   </bookViews>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4922" uniqueCount="1670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4923" uniqueCount="1670">
   <si>
     <t>S. No</t>
   </si>
@@ -12403,7 +12403,9 @@
         <v>1267</v>
       </c>
       <c r="AA87" s="5"/>
-      <c r="AB87" s="5"/>
+      <c r="AB87" s="5" t="s">
+        <v>337</v>
+      </c>
       <c r="AC87" s="5"/>
     </row>
     <row r="88" spans="1:29" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Final latest updated code
</commit_message>
<xml_diff>
--- a/static/uploads/2025-2026/master_sheet.xlsx
+++ b/static/uploads/2025-2026/master_sheet.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/690d49f7c0aa36f5/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pallavai\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="86" documentId="8_{316B5196-EA75-4D10-A879-C2C5EF29FF86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88E5FBE9-19DB-4051-8AA6-8311CF51B208}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF2D40F9-0D87-46DA-BB1C-1AAB67BD5592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9CB53044-4ACA-476F-BD6F-9B67AAF67AA6}"/>
   </bookViews>
@@ -141,7 +141,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4921" uniqueCount="1670">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4923" uniqueCount="1671">
   <si>
     <t>S. No</t>
   </si>
@@ -5151,6 +5151,9 @@
   </si>
   <si>
     <t>AJINKYA SUNIL GAWANDE</t>
+  </si>
+  <si>
+    <t>Google</t>
   </si>
 </sst>
 </file>
@@ -5301,10 +5304,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11705,7 +11704,9 @@
       <c r="Z78" s="2" t="s">
         <v>1260</v>
       </c>
-      <c r="AA78" s="5"/>
+      <c r="AA78" s="5" t="s">
+        <v>1670</v>
+      </c>
       <c r="AB78" s="5"/>
       <c r="AC78" s="5"/>
     </row>
@@ -12483,7 +12484,9 @@
       <c r="Z88" s="2" t="s">
         <v>1268</v>
       </c>
-      <c r="AA88" s="5"/>
+      <c r="AA88" s="5" t="s">
+        <v>1670</v>
+      </c>
       <c r="AB88" s="5"/>
       <c r="AC88" s="5"/>
     </row>

</xml_diff>